<commit_message>
Tracker XLSX: tambah sheet Harian & Mingguan + catat riwayat
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011v1FUP1JSE1oBe6FiKjuY3
</commit_message>
<xml_diff>
--- a/docs/Tracker-Marketing-MD-Heny-Fitriani.xlsx
+++ b/docs/Tracker-Marketing-MD-Heny-Fitriani.xlsx
@@ -10,11 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anggota" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referral" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulanan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Harian" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mingguan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulanan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Anggota'!$A$4:$R$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Harian'!$A$4:$O$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +25,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -102,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,9 +128,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -581,50 +589,64 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4. Rekap – ringkasan otomatis jumlah anggota per status (rumus, jangan diubah).</t>
+          <t>4. Harian – laporan harian ES/BC/BM (diisi tiap hari), rekap mingguan otomatis di sheet Mingguan.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>5. Mingguan – rekap otomatis per anggota dari sheet Harian (rumus).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aturan:</t>
+          <t>6. Rekap – ringkasan otomatis jumlah anggota per status (rumus, jangan diubah).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• Isi hanya sel berlatar krem. Kolom abu/rumus otomatis.</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>• Status: Aktif - Capai Target / Aktif - Belum Capai / Tidak Aktif / Aktivasi Ulang.</t>
+          <t>Aturan:</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>• 1 transaksi jamaah hanya dicatat sekali: di Direct Selling ATAU Referral sesuai atribusi perusahaan.</t>
+          <t>• Isi hanya sel berlatar krem. Kolom abu/rumus otomatis.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• Jabatan: BM, BC, ES. Atasan diisi nama BM/BC langsung.</t>
+          <t>• Status: Aktif - Capai Target / Aktif - Belum Capai / Tidak Aktif / Aktivasi Ulang.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>• 1 transaksi jamaah hanya dicatat sekali: di Direct Selling ATAU Referral sesuai atribusi perusahaan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• Jabatan: BM, BC, ES. Atasan diisi nama BM/BC langsung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>• Kolom 'Evaluasi Ulang' wajib diisi untuk anggota belum capai / tidak aktif.</t>
         </is>
@@ -1992,6 +2014,1077 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LAPORAN HARIAN (ES → BC → BM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>⚠ DATA DUMMY • isi tiap hari, 1 baris per anggota per hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tanggal</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Nama</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Jabatan</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Target Prospek</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Prospek Baru</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Target FU</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Presentasi</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Closing</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Potensi Closing Dekat</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Digital Marketing (post/konten)</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Kendala</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Rencana Besok</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Lapor ke Atasan (jam)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Nur Aisyah</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>19.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Bima Prakoso</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Dewi Lestari</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>19.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Siti Aminah</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Nur Aisyah</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>19.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Bima Prakoso</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="I10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>19.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Dewi Lestari</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="8" t="inlineStr"/>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Siti Aminah</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Nur Aisyah</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="8" t="inlineStr"/>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Bima Prakoso</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="8" t="inlineStr"/>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Dewi Lestari</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>19.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Siti Aminah</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>Prospek belum angkat telp</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>FU prospek panas &amp; presentasi</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:O16"/>
+  <dataValidations count="1">
+    <dataValidation sqref="C5:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BM,BC,ES"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>REKAP MINGGUAN OTOMATIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>⚠ DATA DUMMY • isi tanggal awal &amp; akhir minggu (sel B3, D3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mulai</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>46314</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Akhir</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="n">
+        <v>46320</v>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Nama</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Jabatan</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Prospek Baru</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Calling</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Presentasi</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Closing</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Hari Lapor</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Konversi (Closing/Presentasi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Nur Aisyah</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C5" s="7">
+        <f>SUMIFS(Harian!$E$5:$E$1000,Harian!$B$5:$B$1000,$A5,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="D5" s="7">
+        <f>SUMIFS(Harian!$G$5:$G$1000,Harian!$B$5:$B$1000,$A5,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="E5" s="7">
+        <f>SUMIFS(Harian!$H$5:$H$1000,Harian!$B$5:$B$1000,$A5,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="F5" s="7">
+        <f>SUMIFS(Harian!$I$5:$I$1000,Harian!$B$5:$B$1000,$A5,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="G5" s="7">
+        <f>SUMIFS(Harian!$J$5:$J$1000,Harian!$B$5:$B$1000,$A5,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="H5" s="7">
+        <f>COUNTIFS(Harian!$B$5:$B$1000,$A5,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="I5" s="13">
+        <f>IF(F5=0,0,G5/F5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Bima Prakoso</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C6" s="7">
+        <f>SUMIFS(Harian!$E$5:$E$1000,Harian!$B$5:$B$1000,$A6,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="D6" s="7">
+        <f>SUMIFS(Harian!$G$5:$G$1000,Harian!$B$5:$B$1000,$A6,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="E6" s="7">
+        <f>SUMIFS(Harian!$H$5:$H$1000,Harian!$B$5:$B$1000,$A6,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="F6" s="7">
+        <f>SUMIFS(Harian!$I$5:$I$1000,Harian!$B$5:$B$1000,$A6,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="G6" s="7">
+        <f>SUMIFS(Harian!$J$5:$J$1000,Harian!$B$5:$B$1000,$A6,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="H6" s="7">
+        <f>COUNTIFS(Harian!$B$5:$B$1000,$A6,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="I6" s="13">
+        <f>IF(F6=0,0,G6/F6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Dewi Lestari</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C7" s="7">
+        <f>SUMIFS(Harian!$E$5:$E$1000,Harian!$B$5:$B$1000,$A7,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="D7" s="7">
+        <f>SUMIFS(Harian!$G$5:$G$1000,Harian!$B$5:$B$1000,$A7,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="E7" s="7">
+        <f>SUMIFS(Harian!$H$5:$H$1000,Harian!$B$5:$B$1000,$A7,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="F7" s="7">
+        <f>SUMIFS(Harian!$I$5:$I$1000,Harian!$B$5:$B$1000,$A7,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="G7" s="7">
+        <f>SUMIFS(Harian!$J$5:$J$1000,Harian!$B$5:$B$1000,$A7,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="H7" s="7">
+        <f>COUNTIFS(Harian!$B$5:$B$1000,$A7,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>IF(F7=0,0,G7/F7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Siti Aminah</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C8" s="7">
+        <f>SUMIFS(Harian!$E$5:$E$1000,Harian!$B$5:$B$1000,$A8,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>SUMIFS(Harian!$G$5:$G$1000,Harian!$B$5:$B$1000,$A8,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="E8" s="7">
+        <f>SUMIFS(Harian!$H$5:$H$1000,Harian!$B$5:$B$1000,$A8,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="F8" s="7">
+        <f>SUMIFS(Harian!$I$5:$I$1000,Harian!$B$5:$B$1000,$A8,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="G8" s="7">
+        <f>SUMIFS(Harian!$J$5:$J$1000,Harian!$B$5:$B$1000,$A8,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="H8" s="7">
+        <f>COUNTIFS(Harian!$B$5:$B$1000,$A8,Harian!$A$5:$A$1000,"&gt;="&amp;$B$3,Harian!$A$5:$A$1000,"&lt;="&amp;$D$3)</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>IF(F8=0,0,G8/F8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>(tambah baris &amp; salin rumus untuk anggota lain)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2114,7 +3207,7 @@
         <f>H5-G5</f>
         <v/>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="13">
         <f>IF(G5=0,0,H5/G5)</f>
         <v/>
       </c>
@@ -2159,7 +3252,7 @@
         <f>H6-G6</f>
         <v/>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="13">
         <f>IF(G6=0,0,H6/G6)</f>
         <v/>
       </c>
@@ -2204,7 +3297,7 @@
         <f>H7-G7</f>
         <v/>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="13">
         <f>IF(G7=0,0,H7/G7)</f>
         <v/>
       </c>
@@ -2249,7 +3342,7 @@
         <f>H8-G8</f>
         <v/>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="13">
         <f>IF(G8=0,0,H8/G8)</f>
         <v/>
       </c>
@@ -2290,7 +3383,7 @@
         <f>H9-G9</f>
         <v/>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="13">
         <f>IF(G9=0,0,H9/G9)</f>
         <v/>
       </c>
@@ -2335,7 +3428,7 @@
         <f>H10-G10</f>
         <v/>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="13">
         <f>IF(G10=0,0,H10/G10)</f>
         <v/>
       </c>
@@ -2379,13 +3472,13 @@
         <f>SUM(I5:I10)</f>
         <v/>
       </c>
-      <c r="J11" s="12">
+      <c r="J11" s="15">
         <f>IF(G11=0,0,H11/G11)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Catatan: Total = DS + Referral. Pastikan 1 transaksi tidak dimasukkan di kedua kolom.</t>
         </is>
@@ -2396,7 +3489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2596,7 +3689,7 @@
           <t>% Capai DS</t>
         </is>
       </c>
-      <c r="B13" s="12">
+      <c r="B13" s="15">
         <f>IF(B11=0,0,B12/B11)</f>
         <v/>
       </c>

</xml_diff>